<commit_message>
Update worker summary: propose Julian as contract labor pending CPA review
Julian Budde's single one-time $44 maintenance payment is now shown as
proposed independent contract labor (under $600, no 1099 required) rather
than W-2 wages, with a note flagging the consistency question for the CPA.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018Kdn8Y8BXNQmCYBdY1271v
</commit_message>
<xml_diff>
--- a/2025-worker-payment-summary-for-cpa.xlsx
+++ b/2025-worker-payment-summary-for-cpa.xlsx
@@ -115,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -143,6 +143,9 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -514,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -540,7 +543,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>All four individuals were scheduled and directed by me for work within my rental business; none operate their own established business. I have classified all four as employees pending final confirmation by CPA and legal counsel.</t>
+          <t>Three recurring workers were scheduled and directed by me for work within my rental business and are proposed as employees (W-2). Julian Budde was a single one-time $44 job and is proposed as independent contract labor. All treatment is pending final confirmation by CPA and legal counsel.</t>
         </is>
       </c>
     </row>
@@ -781,12 +784,12 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Equipment maintenance (one-time).</t>
+          <t>Equipment maintenance — single one-time job; no ongoing relationship. See note below.</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>One-time*</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -796,12 +799,12 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Employee</t>
+          <t>Contractor (proposed — CPA to confirm)</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>W-2</t>
+          <t>Contract labor; no 1099 (&lt;$600)</t>
         </is>
       </c>
     </row>
@@ -828,10 +831,18 @@
       <c r="J8" s="8" t="n"/>
       <c r="K8" s="8" t="n"/>
     </row>
+    <row r="10" ht="56" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>* Julian Budde: one payment of $44 for a single equipment-maintenance job, with no ongoing relationship — proposed as independent contract labor (under $600, so no Form 1099-NEC is required). Note for CPA: this is the same category of maintenance work performed by Isaiah and Jeremiah, who are proposed as employees; please confirm that treating Julian's one-time job as contract labor is appropriate and consistent.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A10:K10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1440,18 +1451,18 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="n"/>
-      <c r="B27" s="11" t="inlineStr">
+      <c r="A27" s="11" t="n"/>
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C27" s="12">
+      <c r="C27" s="13">
         <f>SUM(C3:C26)</f>
         <v/>
       </c>
-      <c r="D27" s="10" t="n"/>
-      <c r="E27" s="10" t="n"/>
+      <c r="D27" s="11" t="n"/>
+      <c r="E27" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>